<commit_message>
Auto commit 25-06-2025 17:09:18.81
</commit_message>
<xml_diff>
--- a/GWD Data/GWD DR Abstract.xlsx
+++ b/GWD Data/GWD DR Abstract.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1847" uniqueCount="459">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1877" uniqueCount="466">
   <si>
     <t>GWD Revised Derived Rates 2025 Based on DSR 21/PRICE</t>
   </si>
@@ -1398,6 +1398,27 @@
   </si>
   <si>
     <t>GWDDR369</t>
+  </si>
+  <si>
+    <t>GWDDR370</t>
+  </si>
+  <si>
+    <t>ARS Filter Media</t>
+  </si>
+  <si>
+    <t>GWDDR371</t>
+  </si>
+  <si>
+    <t>GWDDR372</t>
+  </si>
+  <si>
+    <t>GWDDR373</t>
+  </si>
+  <si>
+    <t>GWDDR374</t>
+  </si>
+  <si>
+    <t>GWDDR375</t>
   </si>
 </sst>
 </file>
@@ -1596,7 +1617,7 @@
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1653,9 +1674,6 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="4" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1786,6 +1804,7 @@
       <sheetName val="GWD DR Abstract"/>
       <sheetName val="GWD MR Abstract"/>
       <sheetName val="3 Core Cable PRICE"/>
+      <sheetName val="ARS Filter Media"/>
       <sheetName val="BW Casing Pipes"/>
       <sheetName val="GI on Wall PRICE"/>
       <sheetName val="GI wo Trench"/>
@@ -1861,13 +1880,14 @@
       <sheetData sheetId="35"/>
       <sheetData sheetId="36"/>
       <sheetData sheetId="37"/>
+      <sheetData sheetId="38"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table_1" displayName="Table_1" ref="A3:L372">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table_1" displayName="Table_1" ref="A3:L378">
   <tableColumns count="12">
     <tableColumn id="1" name="Sl No"/>
     <tableColumn id="2" name="Code"/>
@@ -2182,8 +2202,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE87EFAD-0F69-47BA-B0F8-E3A6CAE1B9A6}">
-  <dimension ref="A1:L372"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{166201FD-6B1C-4AE0-9596-BD3E9933B9A6}">
+  <dimension ref="A1:L378"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <sheetData>
     <row r="1" spans="1:12" ht="12.75">
@@ -2315,11 +2335,11 @@
       </c>
       <c r="C5" s="15" t="str">
         <f>'[1]Iron Structure'!A1</f>
-        <v>Estimate  For Fabricated Angle Iron Structure To Support 5000 Litres Capacity Water Tank At 4 m Height</v>
+        <v>Angle Iron Structure To Support 5000 Litres Capacity Water Tank At 4 m Height</v>
       </c>
       <c r="D5" s="15" t="str">
         <f>CONCATENATE(C5," (Code: ",B5,")")</f>
-        <v>Estimate  For Fabricated Angle Iron Structure To Support 5000 Litres Capacity Water Tank At 4 m Height (Code: GWDDR002)</v>
+        <v>Angle Iron Structure To Support 5000 Litres Capacity Water Tank At 4 m Height (Code: GWDDR002)</v>
       </c>
       <c r="E5" s="14" t="s">
         <v>17</v>
@@ -2358,11 +2378,11 @@
       </c>
       <c r="C6" s="15" t="str">
         <f>'[1]Iron Structure'!A44</f>
-        <v>Estimate  For Fabricated Angle Iron Structure To Support 3000 Litres Capacity Water Tank At 4 m Height</v>
+        <v>Angle Iron Structure To Support 3000 Litres Capacity Water Tank At 4 m Height</v>
       </c>
       <c r="D6" s="15" t="str">
         <f>CONCATENATE(C6," (Code: ",B6,")")</f>
-        <v>Estimate  For Fabricated Angle Iron Structure To Support 3000 Litres Capacity Water Tank At 4 m Height (Code: GWDDR003)</v>
+        <v>Angle Iron Structure To Support 3000 Litres Capacity Water Tank At 4 m Height (Code: GWDDR003)</v>
       </c>
       <c r="E6" s="14" t="s">
         <v>17</v>
@@ -2401,11 +2421,11 @@
       </c>
       <c r="C7" s="15" t="str">
         <f>'[1]Iron Structure'!A87</f>
-        <v>Estimate  For Fabricated Angle Iron Structure To Support 5000 Litres Capacity Water Tank At 6 m Height</v>
+        <v>Angle Iron Structure To Support 5000 Litres Capacity Water Tank At 6 m Height</v>
       </c>
       <c r="D7" s="15" t="str">
         <f>CONCATENATE(C7," (Code: ",B7,")")</f>
-        <v>Estimate  For Fabricated Angle Iron Structure To Support 5000 Litres Capacity Water Tank At 6 m Height (Code: GWDDR004)</v>
+        <v>Angle Iron Structure To Support 5000 Litres Capacity Water Tank At 6 m Height (Code: GWDDR004)</v>
       </c>
       <c r="E7" s="14" t="s">
         <v>17</v>
@@ -2444,11 +2464,11 @@
       </c>
       <c r="C8" s="15" t="str">
         <f>'[1]Iron Structure'!A132</f>
-        <v>Estimate  For Fabricated Angle Iron Structure To Support 3000 Litres Capacity Water Tank At 6 m Height</v>
+        <v>Angle Iron Structure To Support 3000 Litres Capacity Water Tank At 6 m Height</v>
       </c>
       <c r="D8" s="15" t="str">
         <f>CONCATENATE(C8," (Code: ",B8,")")</f>
-        <v>Estimate  For Fabricated Angle Iron Structure To Support 3000 Litres Capacity Water Tank At 6 m Height (Code: GWDDR005)</v>
+        <v>Angle Iron Structure To Support 3000 Litres Capacity Water Tank At 6 m Height (Code: GWDDR005)</v>
       </c>
       <c r="E8" s="14" t="s">
         <v>17</v>
@@ -5016,11 +5036,11 @@
       </c>
       <c r="C67" s="15" t="str">
         <f>[1]WTP!B3</f>
-        <v>Supplying, assembling, fibre reinforced polymer vessel (FRP) size  (14" Dia 65" Height) Weight – 21 kg, Tank Volume - 150 liter, Material- Polyethylene, Max Pressure -150 PSI, Max Vacuum- 5" Hg, Max temperature-49'c, Capacity- 1000-10000 L, opening at top &amp; bottom  including hire &amp; labour charges, fittings &amp; accessories etc.complete, as per direction of Engineer-in-charge</v>
+        <v>Supplying, assembling, fibre reinforced polymer vessel (FRP) size  (14" Dia 65" Height) Weight - 21 kg, Tank Volume - 150 liter, Material- Polyethylene, Max Pressure -150 PSI, Max Vacuum- 5" Hg, Max temperature-49'c, Capacity- 1000-10000 L, opening at top &amp; bottom  including hire &amp; labour charges, fittings &amp; accessories etc.complete, as per direction of Engineer-in-charge</v>
       </c>
       <c r="D67" s="15" t="str">
         <f>CONCATENATE(C67," (Code: ",B67,")")</f>
-        <v>Supplying, assembling, fibre reinforced polymer vessel (FRP) size  (14" Dia 65" Height) Weight – 21 kg, Tank Volume - 150 liter, Material- Polyethylene, Max Pressure -150 PSI, Max Vacuum- 5" Hg, Max temperature-49'c, Capacity- 1000-10000 L, opening at top &amp; bottom  including hire &amp; labour charges, fittings &amp; accessories etc.complete, as per direction of Engineer-in-charge  (Code: GWDDR064)</v>
+        <v>Supplying, assembling, fibre reinforced polymer vessel (FRP) size  (14" Dia 65" Height) Weight - 21 kg, Tank Volume - 150 liter, Material- Polyethylene, Max Pressure -150 PSI, Max Vacuum- 5" Hg, Max temperature-49'c, Capacity- 1000-10000 L, opening at top &amp; bottom  including hire &amp; labour charges, fittings &amp; accessories etc.complete, as per direction of Engineer-in-charge  (Code: GWDDR064)</v>
       </c>
       <c r="E67" s="14" t="s">
         <v>17</v>
@@ -5060,11 +5080,11 @@
       </c>
       <c r="C68" s="15" t="str">
         <f>[1]WTP!B17</f>
-        <v>Supplying, assembling, fibre reinforced polymer vessel (FRP) size  (16" Dia 65" Height) Weight – 22 kg, Tank Volume - 185 liter, Material- Polyethylene, Max Pressure -150 PSI, Max Vacuum- 5" Hg, Max temperature-49'c, Capacity- 1000-10000 L, opening at top &amp; bottom  including hire &amp; labour charges, fittings &amp; accessories etc.complete, as per direction of Engineer-in-charge</v>
+        <v>Supplying, assembling, fibre reinforced polymer vessel (FRP) size  (16" Dia 65" Height) Weight - 22 kg, Tank Volume - 185 liter, Material- Polyethylene, Max Pressure -150 PSI, Max Vacuum- 5" Hg, Max temperature-49'c, Capacity- 1000-10000 L, opening at top &amp; bottom  including hire &amp; labour charges, fittings &amp; accessories etc.complete, as per direction of Engineer-in-charge</v>
       </c>
       <c r="D68" s="15" t="str">
         <f>CONCATENATE(C68," (Code: ",B68,")")</f>
-        <v>Supplying, assembling, fibre reinforced polymer vessel (FRP) size  (16" Dia 65" Height) Weight – 22 kg, Tank Volume - 185 liter, Material- Polyethylene, Max Pressure -150 PSI, Max Vacuum- 5" Hg, Max temperature-49'c, Capacity- 1000-10000 L, opening at top &amp; bottom  including hire &amp; labour charges, fittings &amp; accessories etc.complete, as per direction of Engineer-in-charge  (Code: GWDDR065)</v>
+        <v>Supplying, assembling, fibre reinforced polymer vessel (FRP) size  (16" Dia 65" Height) Weight - 22 kg, Tank Volume - 185 liter, Material- Polyethylene, Max Pressure -150 PSI, Max Vacuum- 5" Hg, Max temperature-49'c, Capacity- 1000-10000 L, opening at top &amp; bottom  including hire &amp; labour charges, fittings &amp; accessories etc.complete, as per direction of Engineer-in-charge  (Code: GWDDR065)</v>
       </c>
       <c r="E68" s="14" t="s">
         <v>17</v>
@@ -5324,11 +5344,11 @@
       </c>
       <c r="C74" s="15" t="str">
         <f>[1]WTP!B102</f>
-        <v>Supplying, assembling, manually operated multi port valve 40 NB Material -PVC, Max pressure – 4kg/cm2,   including hire &amp; labour charges, fittings &amp; accessories etc. all complete, as per direction of Engineer-in-charge</v>
+        <v>Supplying, assembling, manually operated multi port valve 40 NB Material -PVC, Max pressure - 4kg/cm2,   including hire &amp; labour charges, fittings &amp; accessories etc. all complete, as per direction of Engineer-in-charge</v>
       </c>
       <c r="D74" s="15" t="str">
         <f>CONCATENATE(C74," (Code: ",B74,")")</f>
-        <v>Supplying, assembling, manually operated multi port valve 40 NB Material -PVC, Max pressure – 4kg/cm2,   including hire &amp; labour charges, fittings &amp; accessories etc. all complete, as per direction of Engineer-in-charge (Code: GWDDR071)</v>
+        <v>Supplying, assembling, manually operated multi port valve 40 NB Material -PVC, Max pressure - 4kg/cm2,   including hire &amp; labour charges, fittings &amp; accessories etc. all complete, as per direction of Engineer-in-charge (Code: GWDDR071)</v>
       </c>
       <c r="E74" s="14" t="s">
         <v>17</v>
@@ -5368,11 +5388,11 @@
       </c>
       <c r="C75" s="15" t="str">
         <f>[1]WTP!B115</f>
-        <v>Supplying, assembling, manually operated multi port valve flower type 50NB Material -PVC, Max pressure – 4kg/cm2,   including hire &amp; labour charges, fittings &amp; accessories etc. all complete, as per direction of Engineer-in-charge</v>
+        <v>Supplying, assembling, manually operated multi port valve flower type 50NB Material -PVC, Max pressure - 4kg/cm2,   including hire &amp; labour charges, fittings &amp; accessories etc. all complete, as per direction of Engineer-in-charge</v>
       </c>
       <c r="D75" s="15" t="str">
         <f>CONCATENATE(C75," (Code: ",B75,")")</f>
-        <v>Supplying, assembling, manually operated multi port valve flower type 50NB Material -PVC, Max pressure – 4kg/cm2,   including hire &amp; labour charges, fittings &amp; accessories etc. all complete, as per direction of Engineer-in-charge (Code: GWDDR072)</v>
+        <v>Supplying, assembling, manually operated multi port valve flower type 50NB Material -PVC, Max pressure - 4kg/cm2,   including hire &amp; labour charges, fittings &amp; accessories etc. all complete, as per direction of Engineer-in-charge (Code: GWDDR072)</v>
       </c>
       <c r="E75" s="14" t="s">
         <v>17</v>
@@ -5412,11 +5432,11 @@
       </c>
       <c r="C76" s="15" t="str">
         <f>[1]WTP!B128</f>
-        <v>Supplying, assembling, multi port valve 65 NB Manually Material -PVC, Max pressure – 4kg/cm2,   including hire &amp; labour charges, fittings &amp; accessories etc. all complete, as per direction of Engineer-in-charge including hire &amp; labour charges, fittings &amp; accessories etc. all complete, as per direction of Engineer-in-charge</v>
+        <v>Supplying, assembling, multi port valve 65 NB Manually Material -PVC, Max pressure - 4kg/cm2,   including hire &amp; labour charges, fittings &amp; accessories etc. all complete, as per direction of Engineer-in-charge including hire &amp; labour charges, fittings &amp; accessories etc. all complete, as per direction of Engineer-in-charge</v>
       </c>
       <c r="D76" s="15" t="str">
         <f>CONCATENATE(C76," (Code: ",B76,")")</f>
-        <v>Supplying, assembling, multi port valve 65 NB Manually Material -PVC, Max pressure – 4kg/cm2,   including hire &amp; labour charges, fittings &amp; accessories etc. all complete, as per direction of Engineer-in-charge including hire &amp; labour charges, fittings &amp; accessories etc. all complete, as per direction of Engineer-in-charge (Code: GWDDR073)</v>
+        <v>Supplying, assembling, multi port valve 65 NB Manually Material -PVC, Max pressure - 4kg/cm2,   including hire &amp; labour charges, fittings &amp; accessories etc. all complete, as per direction of Engineer-in-charge including hire &amp; labour charges, fittings &amp; accessories etc. all complete, as per direction of Engineer-in-charge (Code: GWDDR073)</v>
       </c>
       <c r="E76" s="14" t="s">
         <v>17</v>
@@ -10199,11 +10219,11 @@
       </c>
       <c r="C185" s="15" t="str">
         <f>'[1]PVC With Trench PRICE'!A3</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge 15 mm dia 12Kfg/cm2 (50.18.9.1.1)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge 15 mm dia 12Kfg/cm2 (50.18.9.1.1)</v>
       </c>
       <c r="D185" s="15" t="str">
         <f>CONCATENATE(C185," (Code: ",B185,")")</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge 15 mm dia 12Kfg/cm2 (50.18.9.1.1) (Code: GWDDR182)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge 15 mm dia 12Kfg/cm2 (50.18.9.1.1) (Code: GWDDR182)</v>
       </c>
       <c r="E185" s="14" t="s">
         <v>28</v>
@@ -10243,11 +10263,11 @@
       </c>
       <c r="C186" s="15" t="str">
         <f>'[1]PVC With Trench PRICE'!A33</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge. 15 mm dia 10Kgf/cm2 (50.18.9.1.2)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge. 15 mm dia 10Kgf/cm2 (50.18.9.1.2)</v>
       </c>
       <c r="D186" s="15" t="str">
         <f>CONCATENATE(C186," (Code: ",B186,")")</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge. 15 mm dia 10Kgf/cm2 (50.18.9.1.2) (Code: GWDDR183)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge. 15 mm dia 10Kgf/cm2 (50.18.9.1.2) (Code: GWDDR183)</v>
       </c>
       <c r="E186" s="14" t="s">
         <v>28</v>
@@ -10287,11 +10307,11 @@
       </c>
       <c r="C187" s="15" t="str">
         <f>'[1]PVC With Trench PRICE'!A63</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints as per direction of Engineer in Charge.20 mm dia 12 Kgf/cm2 (50.18.9.2.1)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints as per direction of Engineer in Charge.20 mm dia 12 Kgf/cm2 (50.18.9.2.1)</v>
       </c>
       <c r="D187" s="15" t="str">
         <f>CONCATENATE(C187," (Code: ",B187,")")</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints as per direction of Engineer in Charge.20 mm dia 12 Kgf/cm2 (50.18.9.2.1) (Code: GWDDR184)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints as per direction of Engineer in Charge.20 mm dia 12 Kgf/cm2 (50.18.9.2.1) (Code: GWDDR184)</v>
       </c>
       <c r="E187" s="14" t="s">
         <v>28</v>
@@ -10331,11 +10351,11 @@
       </c>
       <c r="C188" s="15" t="str">
         <f>'[1]PVC With Trench PRICE'!A93</f>
-        <v>Providing and fixing PVC pipes includings of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge. 20 mm dia 10 Kgf/cm2 (50.18.9.2.2)</v>
+        <v>Providing and fixing PVC pipes including of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge. 20 mm dia 10 Kgf/cm2 (50.18.9.2.2)</v>
       </c>
       <c r="D188" s="15" t="str">
         <f>CONCATENATE(C188," (Code: ",B188,")")</f>
-        <v>Providing and fixing PVC pipes includings of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge. 20 mm dia 10 Kgf/cm2 (50.18.9.2.2) (Code: GWDDR185)</v>
+        <v>Providing and fixing PVC pipes including of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge. 20 mm dia 10 Kgf/cm2 (50.18.9.2.2) (Code: GWDDR185)</v>
       </c>
       <c r="E188" s="14" t="s">
         <v>28</v>
@@ -10375,11 +10395,11 @@
       </c>
       <c r="C189" s="15" t="str">
         <f>'[1]PVC With Trench PRICE'!A123</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge 25 mm dia 12Kfg/cm2 (50.18.9.3.1)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge 25 mm dia 12Kfg/cm2 (50.18.9.3.1)</v>
       </c>
       <c r="D189" s="15" t="str">
         <f>CONCATENATE(C189," (Code: ",B189,")")</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge 25 mm dia 12Kfg/cm2 (50.18.9.3.1) (Code: GWDDR186)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge 25 mm dia 12Kfg/cm2 (50.18.9.3.1) (Code: GWDDR186)</v>
       </c>
       <c r="E189" s="14" t="s">
         <v>28</v>
@@ -10463,11 +10483,11 @@
       </c>
       <c r="C191" s="15" t="str">
         <f>'[1]PVC With Trench PRICE'!A183</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge.32 mm dia 10.Kgf/cm2 (50.18.9.4.1)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge.32 mm dia 10.Kgf/cm2 (50.18.9.4.1)</v>
       </c>
       <c r="D191" s="15" t="str">
         <f>CONCATENATE(C191," (Code: ",B191,")")</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge.32 mm dia 10.Kgf/cm2 (50.18.9.4.1) (Code: GWDDR188)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge.32 mm dia 10.Kgf/cm2 (50.18.9.4.1) (Code: GWDDR188)</v>
       </c>
       <c r="E191" s="14" t="s">
         <v>28</v>
@@ -10507,11 +10527,11 @@
       </c>
       <c r="C192" s="15" t="str">
         <f>'[1]PVC With Trench PRICE'!A213</f>
-        <v>Providing and fixing PVC pipes includings joints of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge. 32 mm dia 6 Kgf/cm2 (50.18.9.4.2)</v>
+        <v>Providing and fixing PVC pipes including joints of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge. 32 mm dia 6 Kgf/cm2 (50.18.9.4.2)</v>
       </c>
       <c r="D192" s="15" t="str">
         <f>CONCATENATE(C192," (Code: ",B192,")")</f>
-        <v>Providing and fixing PVC pipes includings joints of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge. 32 mm dia 6 Kgf/cm2 (50.18.9.4.2) (Code: GWDDR189)</v>
+        <v>Providing and fixing PVC pipes including joints of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge. 32 mm dia 6 Kgf/cm2 (50.18.9.4.2) (Code: GWDDR189)</v>
       </c>
       <c r="E192" s="14" t="s">
         <v>28</v>
@@ -10551,11 +10571,11 @@
       </c>
       <c r="C193" s="15" t="str">
         <f>'[1]PVC With Trench PRICE'!A243</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step PVC solvent cement, trenching refilling &amp; testing of joints complete as per direction of Engineer in Charge 40 mm dia 10Kgf/cm2 (50.18.9.5.1)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step PVC solvent cement, trenching refilling &amp; testing of joints complete as per direction of Engineer in Charge 40 mm dia 10Kgf/cm2 (50.18.9.5.1)</v>
       </c>
       <c r="D193" s="15" t="str">
         <f>CONCATENATE(C193," (Code: ",B193,")")</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step PVC solvent cement, trenching refilling &amp; testing of joints complete as per direction of Engineer in Charge 40 mm dia 10Kgf/cm2 (50.18.9.5.1) (Code: GWDDR190)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step PVC solvent cement, trenching refilling &amp; testing of joints complete as per direction of Engineer in Charge 40 mm dia 10Kgf/cm2 (50.18.9.5.1) (Code: GWDDR190)</v>
       </c>
       <c r="E193" s="14" t="s">
         <v>28</v>
@@ -10595,11 +10615,11 @@
       </c>
       <c r="C194" s="15" t="str">
         <f>'[1]PVC With Trench PRICE'!A273</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints compete as per direction of Engineer in Charge. 40 mm dia 6 Kgf/cm2 (50.18.9.5.2)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints compete as per direction of Engineer in Charge. 40 mm dia 6 Kgf/cm2 (50.18.9.5.2)</v>
       </c>
       <c r="D194" s="15" t="str">
         <f>CONCATENATE(C194," (Code: ",B194,")")</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints compete as per direction of Engineer in Charge. 40 mm dia 6 Kgf/cm2 (50.18.9.5.2) (Code: GWDDR191)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints compete as per direction of Engineer in Charge. 40 mm dia 6 Kgf/cm2 (50.18.9.5.2) (Code: GWDDR191)</v>
       </c>
       <c r="E194" s="14" t="s">
         <v>28</v>
@@ -10639,11 +10659,11 @@
       </c>
       <c r="C195" s="15" t="str">
         <f>'[1]PVC With Trench PRICE'!A303</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge. 50 mm dia 10Kgf/cm2 (50.18.9.6.1)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge. 50 mm dia 10Kgf/cm2 (50.18.9.6.1)</v>
       </c>
       <c r="D195" s="15" t="str">
         <f>CONCATENATE(C195," (Code: ",B195,")")</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge. 50 mm dia 10Kgf/cm2 (50.18.9.6.1) (Code: GWDDR192)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge. 50 mm dia 10Kgf/cm2 (50.18.9.6.1) (Code: GWDDR192)</v>
       </c>
       <c r="E195" s="14" t="s">
         <v>28</v>
@@ -10683,11 +10703,11 @@
       </c>
       <c r="C196" s="15" t="str">
         <f>'[1]PVC With Trench PRICE'!A333</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge. 50 mm dia 6 Kgf/cm2 (50.18.9.6.2)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge. 50 mm dia 6 Kgf/cm2 (50.18.9.6.2)</v>
       </c>
       <c r="D196" s="15" t="str">
         <f>CONCATENATE(C196," (Code: ",B196,")")</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge. 50 mm dia 6 Kgf/cm2 (50.18.9.6.2) (Code: GWDDR193)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge. 50 mm dia 6 Kgf/cm2 (50.18.9.6.2) (Code: GWDDR193)</v>
       </c>
       <c r="E196" s="14" t="s">
         <v>28</v>
@@ -10727,11 +10747,11 @@
       </c>
       <c r="C197" s="15" t="str">
         <f>'[1]PVC With Trench PRICE'!A363</f>
-        <v>Providing and fixing PVC pipes includings of pipes with one step PVC solvent cement, trenching refilling &amp; testing of joints complete as per direction of Engineer in Charge. 63 mm dia 6Kgf/cm2 (50.18.9.7.1)</v>
+        <v>Providing and fixing PVC pipes including of pipes with one step PVC solvent cement, trenching refilling &amp; testing of joints complete as per direction of Engineer in Charge. 63 mm dia 6Kgf/cm2 (50.18.9.7.1)</v>
       </c>
       <c r="D197" s="15" t="str">
         <f>CONCATENATE(C197," (Code: ",B197,")")</f>
-        <v>Providing and fixing PVC pipes includings of pipes with one step PVC solvent cement, trenching refilling &amp; testing of joints complete as per direction of Engineer in Charge. 63 mm dia 6Kgf/cm2 (50.18.9.7.1) (Code: GWDDR194)</v>
+        <v>Providing and fixing PVC pipes including of pipes with one step PVC solvent cement, trenching refilling &amp; testing of joints complete as per direction of Engineer in Charge. 63 mm dia 6Kgf/cm2 (50.18.9.7.1) (Code: GWDDR194)</v>
       </c>
       <c r="E197" s="14" t="s">
         <v>28</v>
@@ -10771,11 +10791,11 @@
       </c>
       <c r="C198" s="15" t="str">
         <f>'[1]PVC With Trench PRICE'!A393</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge.63 mm dia 4 Kgf/cm2 (50.18.9.7.2)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge.63 mm dia 4 Kgf/cm2 (50.18.9.7.2)</v>
       </c>
       <c r="D198" s="15" t="str">
         <f>CONCATENATE(C198," (Code: ",B198,")")</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge.63 mm dia 4 Kgf/cm2 (50.18.9.7.2) (Code: GWDDR195)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge.63 mm dia 4 Kgf/cm2 (50.18.9.7.2) (Code: GWDDR195)</v>
       </c>
       <c r="E198" s="14" t="s">
         <v>28</v>
@@ -10815,11 +10835,11 @@
       </c>
       <c r="C199" s="15" t="str">
         <f>'[1]PVC With Trench PRICE'!A423</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge. 75 mm dia 6 Kgf/ cm2 50.18.9.8.1)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge. 75 mm dia 6 Kgf/ cm2 50.18.9.8.1)</v>
       </c>
       <c r="D199" s="15" t="str">
         <f>CONCATENATE(C199," (Code: ",B199,")")</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge. 75 mm dia 6 Kgf/ cm2 50.18.9.8.1) (Code: GWDDR196)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of joints complete as per direction of Engineer in Charge. 75 mm dia 6 Kgf/ cm2 50.18.9.8.1) (Code: GWDDR196)</v>
       </c>
       <c r="E199" s="14" t="s">
         <v>28</v>
@@ -10859,11 +10879,11 @@
       </c>
       <c r="C200" s="15" t="str">
         <f>'[1]PVC With Trench PRICE'!A453</f>
-        <v>Providing and fixing PVC pipes includings of pipes with one step PVC solvent cement, trenching and refilling &amp; testing of joints complete as per direction of Engineer in Charge. 75 mm dia 4 Kgf/cm2 50.18.9.8.2)</v>
+        <v>Providing and fixing PVC pipes including of pipes with one step PVC solvent cement, trenching and refilling &amp; testing of joints complete as per direction of Engineer in Charge. 75 mm dia 4 Kgf/cm2 50.18.9.8.2)</v>
       </c>
       <c r="D200" s="15" t="str">
         <f>CONCATENATE(C200," (Code: ",B200,")")</f>
-        <v>Providing and fixing PVC pipes includings of pipes with one step PVC solvent cement, trenching and refilling &amp; testing of joints complete as per direction of Engineer in Charge. 75 mm dia 4 Kgf/cm2 50.18.9.8.2) (Code: GWDDR197)</v>
+        <v>Providing and fixing PVC pipes including of pipes with one step PVC solvent cement, trenching and refilling &amp; testing of joints complete as per direction of Engineer in Charge. 75 mm dia 4 Kgf/cm2 50.18.9.8.2) (Code: GWDDR197)</v>
       </c>
       <c r="E200" s="14" t="s">
         <v>28</v>
@@ -10903,11 +10923,11 @@
       </c>
       <c r="C201" s="15" t="str">
         <f>'[1]PVC With Trench PRICE'!A483</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of Joints complete as per direction of engineer in charge.110 mm dia 6Kgf/cm2 (50.18.9.9.1)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of Joints complete as per direction of engineer in charge.110 mm dia 6Kgf/cm2 (50.18.9.9.1)</v>
       </c>
       <c r="D201" s="15" t="str">
         <f>CONCATENATE(C201," (Code: ",B201,")")</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of Joints complete as per direction of engineer in charge.110 mm dia 6Kgf/cm2 (50.18.9.9.1) (Code: GWDDR198)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step PVC solvent cement, trenching, refilling &amp; testing of Joints complete as per direction of engineer in charge.110 mm dia 6Kgf/cm2 (50.18.9.9.1) (Code: GWDDR198)</v>
       </c>
       <c r="E201" s="14" t="s">
         <v>28</v>
@@ -10991,11 +11011,11 @@
       </c>
       <c r="C203" s="15" t="str">
         <f>'[1]PVC With Trench PRICE'!A543</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step pvc solvent cement, trenching , refilling &amp; testing of joints complete as per direction of Engineer in Charge. 150 mm dia 6 Kgf/cm2 (50.18.9.10.1)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step pvc solvent cement, trenching , refilling &amp; testing of joints complete as per direction of Engineer in Charge. 150 mm dia 6 Kgf/cm2 (50.18.9.10.1)</v>
       </c>
       <c r="D203" s="15" t="str">
         <f>CONCATENATE(C203," (Code: ",B203,")")</f>
-        <v>Providing and fixing PVC pipes includings jointing of pipes with one step pvc solvent cement, trenching , refilling &amp; testing of joints complete as per direction of Engineer in Charge. 150 mm dia 6 Kgf/cm2 (50.18.9.10.1) (Code: GWDDR200)</v>
+        <v>Providing and fixing PVC pipes including jointing of pipes with one step pvc solvent cement, trenching , refilling &amp; testing of joints complete as per direction of Engineer in Charge. 150 mm dia 6 Kgf/cm2 (50.18.9.10.1) (Code: GWDDR200)</v>
       </c>
       <c r="E203" s="14" t="s">
         <v>28</v>
@@ -18226,10 +18246,10 @@
       <c r="F370" s="16" t="s">
         <v>18</v>
       </c>
-      <c r="G370" s="24" t="s">
+      <c r="G370" s="19" t="s">
         <v>456</v>
       </c>
-      <c r="H370" s="24" t="s">
+      <c r="H370" s="19" t="s">
         <v>157</v>
       </c>
       <c r="I370" s="14">
@@ -18334,6 +18354,264 @@
       <c r="L372" s="16">
         <f>SUM(I372:K372)</f>
         <v>3067.1952670000001</v>
+      </c>
+    </row>
+    <row r="373" spans="1:12" ht="12.75">
+      <c r="A373" s="14">
+        <v>370</v>
+      </c>
+      <c r="B373" s="15" t="s">
+        <v>459</v>
+      </c>
+      <c r="C373" s="15" t="str">
+        <f>'[1]ARS Filter Media'!B2</f>
+        <v>Supply and filling of 40mm metal as filter medium</v>
+      </c>
+      <c r="D373" s="15" t="str">
+        <f>CONCATENATE(C373," (Code: ",B373,")")</f>
+        <v>Supply and filling of 40mm metal as filter medium (Code: GWDDR370)</v>
+      </c>
+      <c r="E373" s="18" t="s">
+        <v>320</v>
+      </c>
+      <c r="F373" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="G373" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="H373" s="19" t="s">
+        <v>460</v>
+      </c>
+      <c r="I373" s="14">
+        <v>0</v>
+      </c>
+      <c r="J373" s="16">
+        <f>'[1]ARS Filter Media'!F16</f>
+        <v>2016.60</v>
+      </c>
+      <c r="K373" s="16">
+        <f>J373*($L$2-1)</f>
+        <v>896.37869999999998</v>
+      </c>
+      <c r="L373" s="16">
+        <f>SUM(I373:K373)</f>
+        <v>2912.9787000000001</v>
+      </c>
+    </row>
+    <row r="374" spans="1:12" ht="12.75">
+      <c r="A374" s="14">
+        <v>371</v>
+      </c>
+      <c r="B374" s="15" t="s">
+        <v>461</v>
+      </c>
+      <c r="C374" s="15" t="str">
+        <f>'[1]ARS Filter Media'!B18</f>
+        <v>Supply and filling of 25mm metal as filter medium</v>
+      </c>
+      <c r="D374" s="15" t="str">
+        <f>CONCATENATE(C374," (Code: ",B374,")")</f>
+        <v>Supply and filling of 25mm metal as filter medium (Code: GWDDR371)</v>
+      </c>
+      <c r="E374" s="18" t="s">
+        <v>320</v>
+      </c>
+      <c r="F374" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="G374" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="H374" s="19" t="s">
+        <v>460</v>
+      </c>
+      <c r="I374" s="14">
+        <v>0</v>
+      </c>
+      <c r="J374" s="16">
+        <f>'[1]ARS Filter Media'!F32</f>
+        <v>2058.10</v>
+      </c>
+      <c r="K374" s="16">
+        <f>J374*($L$2-1)</f>
+        <v>914.82545000000005</v>
+      </c>
+      <c r="L374" s="16">
+        <f>SUM(I374:K374)</f>
+        <v>2972.9254500000002</v>
+      </c>
+    </row>
+    <row r="375" spans="1:12" ht="12.75">
+      <c r="A375" s="14">
+        <v>372</v>
+      </c>
+      <c r="B375" s="15" t="s">
+        <v>462</v>
+      </c>
+      <c r="C375" s="15" t="str">
+        <f>'[1]ARS Filter Media'!B34</f>
+        <v>Supply and filling of 20mm/6mm metal as filter medium</v>
+      </c>
+      <c r="D375" s="15" t="str">
+        <f>CONCATENATE(C375," (Code: ",B375,")")</f>
+        <v>Supply and filling of 20mm/6mm metal as filter medium (Code: GWDDR372)</v>
+      </c>
+      <c r="E375" s="18" t="s">
+        <v>320</v>
+      </c>
+      <c r="F375" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="G375" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="H375" s="19" t="s">
+        <v>460</v>
+      </c>
+      <c r="I375" s="14">
+        <v>0</v>
+      </c>
+      <c r="J375" s="16">
+        <f>'[1]ARS Filter Media'!F48</f>
+        <v>2116.15</v>
+      </c>
+      <c r="K375" s="16">
+        <f>J375*($L$2-1)</f>
+        <v>940.62867500000004</v>
+      </c>
+      <c r="L375" s="16">
+        <f>SUM(I375:K375)</f>
+        <v>3056.778675</v>
+      </c>
+    </row>
+    <row r="376" spans="1:12" ht="12.75">
+      <c r="A376" s="14">
+        <v>373</v>
+      </c>
+      <c r="B376" s="15" t="s">
+        <v>463</v>
+      </c>
+      <c r="C376" s="15" t="str">
+        <f>'[1]ARS Filter Media'!B50</f>
+        <v>Supply and filling of Coarse Sand as filter medium</v>
+      </c>
+      <c r="D376" s="15" t="str">
+        <f>CONCATENATE(C376," (Code: ",B376,")")</f>
+        <v>Supply and filling of Coarse Sand as filter medium (Code: GWDDR373)</v>
+      </c>
+      <c r="E376" s="18" t="s">
+        <v>320</v>
+      </c>
+      <c r="F376" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="G376" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="H376" s="19" t="s">
+        <v>460</v>
+      </c>
+      <c r="I376" s="14">
+        <v>0</v>
+      </c>
+      <c r="J376" s="16">
+        <f>'[1]ARS Filter Media'!F64</f>
+        <v>2382.15</v>
+      </c>
+      <c r="K376" s="16">
+        <f>J376*($L$2-1)</f>
+        <v>1058.865675</v>
+      </c>
+      <c r="L376" s="16">
+        <f>SUM(I376:K376)</f>
+        <v>3441.0156750000001</v>
+      </c>
+    </row>
+    <row r="377" spans="1:12" ht="12.75">
+      <c r="A377" s="14">
+        <v>374</v>
+      </c>
+      <c r="B377" s="15" t="s">
+        <v>464</v>
+      </c>
+      <c r="C377" s="15" t="str">
+        <f>'[1]ARS Filter Media'!B66</f>
+        <v>Supply and filling of Charcoal as filter medium</v>
+      </c>
+      <c r="D377" s="15" t="str">
+        <f>CONCATENATE(C377," (Code: ",B377,")")</f>
+        <v>Supply and filling of Charcoal as filter medium (Code: GWDDR374)</v>
+      </c>
+      <c r="E377" s="18" t="s">
+        <v>320</v>
+      </c>
+      <c r="F377" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="G377" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="H377" s="19" t="s">
+        <v>460</v>
+      </c>
+      <c r="I377" s="14">
+        <v>0</v>
+      </c>
+      <c r="J377" s="16">
+        <f>'[1]ARS Filter Media'!F82</f>
+        <v>2510.45</v>
+      </c>
+      <c r="K377" s="16">
+        <f>J377*($L$2-1)</f>
+        <v>1115.895025</v>
+      </c>
+      <c r="L377" s="16">
+        <f>SUM(I377:K377)</f>
+        <v>3626.3450250000001</v>
+      </c>
+    </row>
+    <row r="378" spans="1:12" ht="12.75">
+      <c r="A378" s="14">
+        <v>375</v>
+      </c>
+      <c r="B378" s="15" t="s">
+        <v>465</v>
+      </c>
+      <c r="C378" s="15" t="str">
+        <f>[1]Services!B19</f>
+        <v>Rotary cum DTH OB Drilling</v>
+      </c>
+      <c r="D378" s="15" t="str">
+        <f>CONCATENATE(C378," (Code: ",B378,")")</f>
+        <v>Rotary cum DTH OB Drilling (Code: GWDDR375)</v>
+      </c>
+      <c r="E378" s="23" t="s">
+        <v>28</v>
+      </c>
+      <c r="F378" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="G378" s="19" t="s">
+        <v>456</v>
+      </c>
+      <c r="H378" s="19" t="s">
+        <v>157</v>
+      </c>
+      <c r="I378" s="14">
+        <f>[1]Services!D19</f>
+        <v>1985</v>
+      </c>
+      <c r="J378" s="14">
+        <v>0</v>
+      </c>
+      <c r="K378" s="16">
+        <f>J378*($L$2-1)</f>
+        <v>0</v>
+      </c>
+      <c r="L378" s="16">
+        <f>SUM(I378:K378)</f>
+        <v>1985</v>
       </c>
     </row>
   </sheetData>

</xml_diff>